<commit_message>
Update daily work log
</commit_message>
<xml_diff>
--- a/Enpro-Daily-Work-Log.xlsx
+++ b/Enpro-Daily-Work-Log.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="155">
   <si>
     <t>Date</t>
   </si>
@@ -243,6 +243,99 @@
     <t>Enpro-Daily-Work-Log.xlsx</t>
   </si>
   <si>
+    <t>Evening</t>
+  </si>
+  <si>
+    <t>Viewport-aware typography</t>
+  </si>
+  <si>
+    <t>Fluid type now scales with screen height as well as width, so wide-but-short screens no longer push sections past the fold</t>
+  </si>
+  <si>
+    <t>tailwind.config.ts</t>
+  </si>
+  <si>
+    <t>Landing page sections fitted to screen</t>
+  </si>
+  <si>
+    <t>Image and card heights capped in vh, spacing tightened, scroll indicator no longer overlaps buttons</t>
+  </si>
+  <si>
+    <t>All landing sections</t>
+  </si>
+  <si>
+    <t>Detail pages fitted to screen</t>
+  </si>
+  <si>
+    <t>Every section on the About Us and service pages made full-height and vertically centred; container widths fixed</t>
+  </si>
+  <si>
+    <t>AboutUs.tsx, ServiceDetail.tsx</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Project Impact section redesigned</t>
+  </si>
+  <si>
+    <t>Cards replaced with outlined numerals on a stepped baseline, separated by hairlines - a distinct third concept</t>
+  </si>
+  <si>
+    <t>Other Services section redesigned</t>
+  </si>
+  <si>
+    <t>Chips replaced with an index list; each row sweeps in the brand colour and reveals that service's artwork on hover</t>
+  </si>
+  <si>
+    <t>How We Work section restyled</t>
+  </si>
+  <si>
+    <t>Dark canvas with grid texture, outlined numerals and a growing accent bar on hover</t>
+  </si>
+  <si>
+    <t>Capability strip separated</t>
+  </si>
+  <si>
+    <t>Moved into its own compact dark band so the What We Do section clears one screen</t>
+  </si>
+  <si>
+    <t>Call-to-action redesigned</t>
+  </si>
+  <si>
+    <t>Plain grey band replaced with a dark card using the client photograph, brand glow and a direct email link</t>
+  </si>
+  <si>
+    <t>404 page rebranded</t>
+  </si>
+  <si>
+    <t>Default template page replaced with a branded dark page matching the rest of the site</t>
+  </si>
+  <si>
+    <t>src/pages/NotFound.tsx</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>All three client documents re-verified</t>
+  </si>
+  <si>
+    <t>Landing Page, About Us and Services-01 checked line by line against the build; all content confirmed accurate</t>
+  </si>
+  <si>
+    <t>Delivery</t>
+  </si>
+  <si>
+    <t>Work committed and pushed</t>
+  </si>
+  <si>
+    <t>59 files committed and pushed to the main branch - first commit since 16 May 2026</t>
+  </si>
+  <si>
+    <t>github.com/msohaiilkz/enpro</t>
+  </si>
+  <si>
     <t>Sessions</t>
   </si>
   <si>
@@ -270,10 +363,13 @@
     <t>No work</t>
   </si>
   <si>
-    <t>1 (afternoon)</t>
-  </si>
-  <si>
-    <t>Work history review and reporting</t>
+    <t>2 (afternoon + evening)</t>
+  </si>
+  <si>
+    <t>Responsive overhaul across every page, three sections redesigned, CTA and 404 rebuilt, all three client documents re-verified, work committed and pushed</t>
+  </si>
+  <si>
+    <t>~85%</t>
   </si>
   <si>
     <t>Item</t>
@@ -282,59 +378,113 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>About Us page review</t>
-  </si>
-  <si>
-    <t>Client-facing review of the rebuilt page</t>
+    <t>Landing page</t>
+  </si>
+  <si>
+    <t>All content and layout instructions from the client document implemented</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>About Us page</t>
+  </si>
+  <si>
+    <t>All three parts built - About Enpro, Built to Evolve, Our Approach</t>
+  </si>
+  <si>
+    <t>Services-01 detail page</t>
+  </si>
+  <si>
+    <t>What We Do, How We Work and Project Impact all built as three distinct concepts</t>
+  </si>
+  <si>
+    <t>Responsive across the site</t>
+  </si>
+  <si>
+    <t>Every page and section verified across resolutions</t>
+  </si>
+  <si>
+    <t>Client confirmations needed</t>
+  </si>
+  <si>
+    <t>Hero buttons removed, 3 cards + Show More, hidden card headings, and two sections we added (Other Services, CTA)</t>
+  </si>
+  <si>
+    <t>To confirm</t>
+  </si>
+  <si>
+    <t>Contact form backend</t>
+  </si>
+  <si>
+    <t>Blocked - waiting on the destination email address</t>
+  </si>
+  <si>
+    <t>Blocked</t>
+  </si>
+  <si>
+    <t>Logo source file</t>
+  </si>
+  <si>
+    <t>Blocked - vector or transparent PNG needed to fix the letter 'o'</t>
+  </si>
+  <si>
+    <t>enpro-logo.png</t>
+  </si>
+  <si>
+    <t>Blocked - imported by TopNavbar but missing; a temporary fallback is in place</t>
+  </si>
+  <si>
+    <t>Social profile URLs</t>
+  </si>
+  <si>
+    <t>Blocked - LinkedIn, Facebook and WhatsApp links are placeholders</t>
+  </si>
+  <si>
+    <t>Phone number and address</t>
+  </si>
+  <si>
+    <t>Blocked - only the email address is available</t>
+  </si>
+  <si>
+    <t>Hero background image</t>
+  </si>
+  <si>
+    <t>Blocked - still the original placeholder</t>
+  </si>
+  <si>
+    <t>Favicon and share image</t>
+  </si>
+  <si>
+    <t>Blocked - still the platform placeholders</t>
+  </si>
+  <si>
+    <t>Remaining five service pages</t>
+  </si>
+  <si>
+    <t>Blocked - waiting on the Services-02 to 06 documents</t>
+  </si>
+  <si>
+    <t>Dead code cleanup</t>
+  </si>
+  <si>
+    <t>Details.jsx, ServiceDetails.jsx, Projects, Counters, Testimonials and unused assets</t>
   </si>
   <si>
     <t>Open</t>
   </si>
   <si>
-    <t>Services detail page - responsive pass</t>
-  </si>
-  <si>
-    <t>Same fluid typography and spacing treatment as the landing and About pages</t>
-  </si>
-  <si>
-    <t>Dead code cleanup</t>
-  </si>
-  <si>
-    <t>Remove Details.jsx, ServiceDetails.jsx, Projects, Counters, Testimonials and unused assets</t>
-  </si>
-  <si>
     <t>Image optimisation</t>
   </si>
   <si>
     <t>about-enpro.jpeg is 519 KB; convert to WebP and add lazy loading</t>
-  </si>
-  <si>
-    <t>Commit the work</t>
-  </si>
-  <si>
-    <t>Nothing has been committed since 16 May 2026</t>
-  </si>
-  <si>
-    <t>Contact form backend</t>
-  </si>
-  <si>
-    <t>Blocked - waiting on the destination email address from the client</t>
-  </si>
-  <si>
-    <t>Blocked</t>
-  </si>
-  <si>
-    <t>Remaining five service pages</t>
-  </si>
-  <si>
-    <t>Blocked - waiting on Services-02 to 06 documents</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -353,6 +503,10 @@
     <font>
       <b/>
       <color rgb="FFBF1E2E"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF15803D"/>
     </font>
   </fonts>
   <fills count="6">
@@ -395,7 +549,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -431,6 +585,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -778,7 +938,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1285,8 +1445,294 @@
         <v>15</v>
       </c>
     </row>
+    <row r="20" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H19"/>
+  <autoFilter ref="A1:H30"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1308,16 +1754,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>76</v>
+        <v>107</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>79</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1325,16 +1771,16 @@
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="C2" s="8">
         <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>82</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1342,16 +1788,16 @@
         <v>59</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="C3" s="12">
         <v>0</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>82</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1359,16 +1805,16 @@
         <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="C4" s="8">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>86</v>
+        <v>117</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>82</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1379,7 +1825,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1389,10 +1835,10 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>119</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -1400,79 +1846,167 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>89</v>
+        <v>121</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>91</v>
+        <v>122</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>91</v>
+        <v>125</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>94</v>
+        <v>126</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>91</v>
+        <v>127</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>96</v>
+        <v>128</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>91</v>
+        <v>129</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>98</v>
+        <v>130</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>99</v>
+        <v>131</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>91</v>
+        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>102</v>
+        <v>134</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>102</v>
+        <v>137</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply client feedback and add new photography
</commit_message>
<xml_diff>
--- a/Enpro-Daily-Work-Log.xlsx
+++ b/Enpro-Daily-Work-Log.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="195">
   <si>
     <t>Date</t>
   </si>
@@ -336,6 +336,126 @@
     <t>github.com/msohaiilkz/enpro</t>
   </si>
   <si>
+    <t>Night</t>
+  </si>
+  <si>
+    <t>Client Changes</t>
+  </si>
+  <si>
+    <t>Heading sizes unified</t>
+  </si>
+  <si>
+    <t>Service page title and category labels brought onto the same two-size scale used across the About Us page</t>
+  </si>
+  <si>
+    <t>ServiceDetail.tsx</t>
+  </si>
+  <si>
+    <t>Services banner title rebuilt</t>
+  </si>
+  <si>
+    <t>The client's artwork carried 'SERVICES' at 1.7x the size and weight of 'ABOUT US'; the lettering was rescaled and thinned inside the image to match exactly</t>
+  </si>
+  <si>
+    <t>banner-services.jpeg</t>
+  </si>
+  <si>
+    <t>Numbers replaced with icons</t>
+  </si>
+  <si>
+    <t>Project Impact, Built to Evolve and Our Approach now use icons that match each item instead of 01-04</t>
+  </si>
+  <si>
+    <t>ServiceDetail.tsx, AboutUs.tsx</t>
+  </si>
+  <si>
+    <t>Eyebrow badges removed</t>
+  </si>
+  <si>
+    <t>The pill labels above the About Us and Why Enpro headings were taken out</t>
+  </si>
+  <si>
+    <t>AboutUs.tsx, Services.tsx</t>
+  </si>
+  <si>
+    <t>Capability strip reworked</t>
+  </si>
+  <si>
+    <t>Label moved on top so each capability fits one line; items numbered and dividers made equal height</t>
+  </si>
+  <si>
+    <t>Word breaks removed site-wide</t>
+  </si>
+  <si>
+    <t>Automatic hyphenation was splitting words across lines; removed everywhere and narrow columns switched to left alignment</t>
+  </si>
+  <si>
+    <t>All sections</t>
+  </si>
+  <si>
+    <t>Navbar fixed with blur</t>
+  </si>
+  <si>
+    <t>The detail-page bar now stays fixed and turns to frosted glass on scroll, compressing slightly</t>
+  </si>
+  <si>
+    <t>TopNavbar.tsx</t>
+  </si>
+  <si>
+    <t>Side menu tidied</t>
+  </si>
+  <si>
+    <t>Address and phone removed leaving only the email, brand icons swapped to the site's own set, logo now links home</t>
+  </si>
+  <si>
+    <t>Service order adjusted</t>
+  </si>
+  <si>
+    <t>Project &amp; Contract Management moved into the default three; Construction Support Services moved to fourth</t>
+  </si>
+  <si>
+    <t>services.ts, Footer.tsx</t>
+  </si>
+  <si>
+    <t>Footer columns balanced</t>
+  </si>
+  <si>
+    <t>Equal-width columns left a large gap after Quick Links; widths now follow the content</t>
+  </si>
+  <si>
+    <t>Footer.tsx</t>
+  </si>
+  <si>
+    <t>Assets</t>
+  </si>
+  <si>
+    <t>New client photography received</t>
+  </si>
+  <si>
+    <t>Seven new images added and mapped to the places they suit</t>
+  </si>
+  <si>
+    <t>src/assets/new images/</t>
+  </si>
+  <si>
+    <t>Hero turned into a slideshow</t>
+  </si>
+  <si>
+    <t>The client's original site photograph stays as the first slide, with the new photography cross-fading behind the tagline</t>
+  </si>
+  <si>
+    <t>Hero.tsx</t>
+  </si>
+  <si>
+    <t>Photograph added to How We Work</t>
+  </si>
+  <si>
+    <t>The service detail page's How We Work column now carries a supporting photograph</t>
+  </si>
+  <si>
+    <t>ServiceDetail.tsx, services.ts</t>
+  </si>
+  <si>
     <t>Sessions</t>
   </si>
   <si>
@@ -363,13 +483,13 @@
     <t>No work</t>
   </si>
   <si>
-    <t>2 (afternoon + evening)</t>
-  </si>
-  <si>
-    <t>Responsive overhaul across every page, three sections redesigned, CTA and 404 rebuilt, all three client documents re-verified, work committed and pushed</t>
-  </si>
-  <si>
-    <t>~85%</t>
+    <t>3 (afternoon, evening, night)</t>
+  </si>
+  <si>
+    <t>Responsive overhaul, three sections redesigned, CTA and 404 rebuilt, documents re-verified, then a full round of client-requested refinements and the new photography put to use</t>
+  </si>
+  <si>
+    <t>~88%</t>
   </si>
   <si>
     <t>Item</t>
@@ -938,7 +1058,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1731,8 +1851,346 @@
         <v>15</v>
       </c>
     </row>
+    <row r="31" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H30"/>
+  <autoFilter ref="A1:H43"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1754,16 +2212,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>107</v>
+        <v>147</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>108</v>
+        <v>148</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>109</v>
+        <v>149</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1771,16 +2229,16 @@
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>111</v>
+        <v>151</v>
       </c>
       <c r="C2" s="8">
         <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>112</v>
+        <v>152</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>113</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1788,16 +2246,16 @@
         <v>59</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>114</v>
+        <v>154</v>
       </c>
       <c r="C3" s="12">
         <v>0</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>115</v>
+        <v>155</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>113</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1805,16 +2263,16 @@
         <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>116</v>
+        <v>156</v>
       </c>
       <c r="C4" s="8">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>117</v>
+        <v>157</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>118</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -1835,10 +2293,10 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>159</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -1846,167 +2304,167 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>121</v>
+        <v>161</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>122</v>
+        <v>162</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>124</v>
+        <v>164</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>125</v>
+        <v>165</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>126</v>
+        <v>166</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>127</v>
+        <v>167</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>128</v>
+        <v>168</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>130</v>
+        <v>170</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>131</v>
+        <v>171</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>132</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>133</v>
+        <v>173</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>134</v>
+        <v>174</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>136</v>
+        <v>176</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>137</v>
+        <v>177</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>138</v>
+        <v>178</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>139</v>
+        <v>179</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>141</v>
+        <v>181</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>142</v>
+        <v>182</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>143</v>
+        <v>183</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>144</v>
+        <v>184</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>145</v>
+        <v>185</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>146</v>
+        <v>186</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>147</v>
+        <v>187</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>148</v>
+        <v>188</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>149</v>
+        <v>189</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>151</v>
+        <v>191</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>152</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>153</v>
+        <v>193</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>154</v>
+        <v>194</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>152</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine side menu, section labels and hero slideshow
</commit_message>
<xml_diff>
--- a/Enpro-Daily-Work-Log.xlsx
+++ b/Enpro-Daily-Work-Log.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="220">
   <si>
     <t>Date</t>
   </si>
@@ -456,6 +456,72 @@
     <t>ServiceDetail.tsx, services.ts</t>
   </si>
   <si>
+    <t>04-Aug-2026</t>
+  </si>
+  <si>
+    <t>Tuesday</t>
+  </si>
+  <si>
+    <t>Late night</t>
+  </si>
+  <si>
+    <t>How We Work numbers replaced</t>
+  </si>
+  <si>
+    <t>The three points now carry icons that match them - compass, workflow and sliders - instead of 01-03</t>
+  </si>
+  <si>
+    <t>Hero slideshow adjusted</t>
+  </si>
+  <si>
+    <t>The aerial port photograph was dropped at the client's request and the BIM workstation photograph added in its place</t>
+  </si>
+  <si>
+    <t>Side menu closing changed</t>
+  </si>
+  <si>
+    <t>The repeated Get a Quote button was replaced with the company tagline, since the button already sits in the top bar</t>
+  </si>
+  <si>
+    <t>Subscribe block removed</t>
+  </si>
+  <si>
+    <t>The newsletter field in the side menu was taken out</t>
+  </si>
+  <si>
+    <t>Side menu order swapped</t>
+  </si>
+  <si>
+    <t>Tagline moved up into a bordered block styled like the site's buttons; social icons moved to the bottom and centred</t>
+  </si>
+  <si>
+    <t>Tagline wording set</t>
+  </si>
+  <si>
+    <t>The menu now closes on 'Engineering Complex Structures. Delivering Certainty.'</t>
+  </si>
+  <si>
+    <t>Section labels differentiated</t>
+  </si>
+  <si>
+    <t>Badges no longer repeat their headings - now 'Our Process' and 'Outcomes Delivered'</t>
+  </si>
+  <si>
+    <t>Keep Exploring badge restyled</t>
+  </si>
+  <si>
+    <t>Brought into the same bordered pill used by every other section label</t>
+  </si>
+  <si>
+    <t>Consistency</t>
+  </si>
+  <si>
+    <t>Button radius audited</t>
+  </si>
+  <si>
+    <t>The last pill-shaped text button (Get a Quote) was squared off; every text button across the site now shares one radius</t>
+  </si>
+  <si>
     <t>Sessions</t>
   </si>
   <si>
@@ -490,6 +556,15 @@
   </si>
   <si>
     <t>~88%</t>
+  </si>
+  <si>
+    <t>1 (late night)</t>
+  </si>
+  <si>
+    <t>A round of client-requested refinements to the side menu, section labels and remaining numbers</t>
+  </si>
+  <si>
+    <t>~89%</t>
   </si>
   <si>
     <t>Item</t>
@@ -1058,7 +1133,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2189,8 +2264,242 @@
         <v>15</v>
       </c>
     </row>
+    <row r="44" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H44" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="H45" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H46" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H47" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H48" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H49" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H50" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H51" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="H52" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H43"/>
+  <autoFilter ref="A1:H52"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2198,7 +2507,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2212,16 +2521,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>149</v>
+        <v>171</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>150</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2229,16 +2538,16 @@
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>151</v>
+        <v>173</v>
       </c>
       <c r="C2" s="8">
         <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>152</v>
+        <v>174</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>153</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2246,16 +2555,16 @@
         <v>59</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
       <c r="C3" s="12">
         <v>0</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>153</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2263,16 +2572,33 @@
         <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="C4" s="8">
         <v>27</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>158</v>
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" s="12">
+        <v>9</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -2293,10 +2619,10 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>159</v>
+        <v>184</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -2304,167 +2630,167 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>161</v>
+        <v>186</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>164</v>
+        <v>189</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>165</v>
+        <v>190</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>166</v>
+        <v>191</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>167</v>
+        <v>192</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>169</v>
+        <v>194</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>163</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>170</v>
+        <v>195</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>171</v>
+        <v>196</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>172</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>173</v>
+        <v>198</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>174</v>
+        <v>199</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>177</v>
+        <v>202</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>178</v>
+        <v>203</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>181</v>
+        <v>206</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>183</v>
+        <v>208</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>184</v>
+        <v>209</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>185</v>
+        <v>210</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>186</v>
+        <v>211</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>187</v>
+        <v>212</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>188</v>
+        <v>213</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>189</v>
+        <v>214</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>191</v>
+        <v>216</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>192</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>193</v>
+        <v>218</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>194</v>
+        <v>219</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>192</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Build all six service detail pages from client documents
</commit_message>
<xml_diff>
--- a/Enpro-Daily-Work-Log.xlsx
+++ b/Enpro-Daily-Work-Log.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="243">
   <si>
     <t>Date</t>
   </si>
@@ -522,6 +522,96 @@
     <t>The last pill-shaped text button (Get a Quote) was squared off; every text button across the site now shares one radius</t>
   </si>
   <si>
+    <t>15-Aug-2026</t>
+  </si>
+  <si>
+    <t>Content</t>
+  </si>
+  <si>
+    <t>Service 02 detail page built</t>
+  </si>
+  <si>
+    <t>Design Review &amp; Value Engineering - four categories, capability strip, approach list and four outcomes, taken from the client's Rev-B document</t>
+  </si>
+  <si>
+    <t>services.ts, ServiceDetail.tsx</t>
+  </si>
+  <si>
+    <t>Service 03 detail page built</t>
+  </si>
+  <si>
+    <t>Construction Support Services - three categories and a four-point approach list</t>
+  </si>
+  <si>
+    <t>src/data/services.ts</t>
+  </si>
+  <si>
+    <t>Service 04 detail page built</t>
+  </si>
+  <si>
+    <t>Project &amp; Contract Management - six categories with lead lines and 47 listed items, plus ten capability entries</t>
+  </si>
+  <si>
+    <t>Service 05 detail page built</t>
+  </si>
+  <si>
+    <t>Environmental &amp; Social Advisory - four categories using the client's own icon set, recoloured from green to the brand red</t>
+  </si>
+  <si>
+    <t>services.ts, icons</t>
+  </si>
+  <si>
+    <t>Service 06 detail page built</t>
+  </si>
+  <si>
+    <t>Digital Engineering &amp; BIM - fourteen capability entries and a 'clients benefit from' list in place of outcome cards</t>
+  </si>
+  <si>
+    <t>Detail page made document-driven</t>
+  </si>
+  <si>
+    <t>The page adapts to each document: 3-6 categories, optional category lead lines, titled points or an approach list, outcome cards or a benefits list, and a per-service capability label</t>
+  </si>
+  <si>
+    <t>Per-service icons</t>
+  </si>
+  <si>
+    <t>Icons moved into the data so each service defines its own, mixing client artwork with line icons</t>
+  </si>
+  <si>
+    <t>Per-service banners</t>
+  </si>
+  <si>
+    <t>Every detail page now opens with its own artwork instead of one shared banner, with the service name set over it</t>
+  </si>
+  <si>
+    <t>PageBanner.tsx, services.ts</t>
+  </si>
+  <si>
+    <t>Banner and photography enlarged</t>
+  </si>
+  <si>
+    <t>Banner height raised to 440px and the service photograph moved out of the sidebar into a full-width band</t>
+  </si>
+  <si>
+    <t>PageBanner.tsx, ServiceDetail.tsx</t>
+  </si>
+  <si>
+    <t>Intro paragraphs unified</t>
+  </si>
+  <si>
+    <t>The tagline and intro were set in two different styles and read as broken lines; they now form a single block</t>
+  </si>
+  <si>
+    <t>Quality</t>
+  </si>
+  <si>
+    <t>Heading levels corrected</t>
+  </si>
+  <si>
+    <t>Each page now carries a single h1 - the service name in the banner - instead of repeating 'What We Do' on every page</t>
+  </si>
+  <si>
     <t>Sessions</t>
   </si>
   <si>
@@ -567,6 +657,15 @@
     <t>~89%</t>
   </si>
   <si>
+    <t>1 (evening)</t>
+  </si>
+  <si>
+    <t>All five remaining service detail pages built from the client's documents, with per-service banners, photography and icons</t>
+  </si>
+  <si>
+    <t>~95%</t>
+  </si>
+  <si>
     <t>Item</t>
   </si>
   <si>
@@ -576,34 +675,22 @@
     <t>Landing page</t>
   </si>
   <si>
-    <t>All content and layout instructions from the client document implemented</t>
-  </si>
-  <si>
     <t>Complete</t>
   </si>
   <si>
     <t>About Us page</t>
   </si>
   <si>
-    <t>All three parts built - About Enpro, Built to Evolve, Our Approach</t>
-  </si>
-  <si>
-    <t>Services-01 detail page</t>
-  </si>
-  <si>
-    <t>What We Do, How We Work and Project Impact all built as three distinct concepts</t>
-  </si>
-  <si>
-    <t>Responsive across the site</t>
-  </si>
-  <si>
-    <t>Every page and section verified across resolutions</t>
-  </si>
-  <si>
-    <t>Client confirmations needed</t>
-  </si>
-  <si>
-    <t>Hero buttons removed, 3 cards + Show More, hidden card headings, and two sections we added (Other Services, CTA)</t>
+    <t>All six service detail pages</t>
+  </si>
+  <si>
+    <t>Built from the client's Rev-B documents</t>
+  </si>
+  <si>
+    <t>Client confirmations</t>
+  </si>
+  <si>
+    <t>Brand red kept for the environmental page, the service order, and the sections we added</t>
   </si>
   <si>
     <t>To confirm</t>
@@ -621,19 +708,13 @@
     <t>Logo source file</t>
   </si>
   <si>
-    <t>Blocked - vector or transparent PNG needed to fix the letter 'o'</t>
-  </si>
-  <si>
-    <t>enpro-logo.png</t>
-  </si>
-  <si>
-    <t>Blocked - imported by TopNavbar but missing; a temporary fallback is in place</t>
+    <t>Blocked - vector or transparent PNG needed</t>
   </si>
   <si>
     <t>Social profile URLs</t>
   </si>
   <si>
-    <t>Blocked - LinkedIn, Facebook and WhatsApp links are placeholders</t>
+    <t>Blocked - all three links are placeholders</t>
   </si>
   <si>
     <t>Phone number and address</t>
@@ -642,37 +723,25 @@
     <t>Blocked - only the email address is available</t>
   </si>
   <si>
-    <t>Hero background image</t>
-  </si>
-  <si>
-    <t>Blocked - still the original placeholder</t>
-  </si>
-  <si>
     <t>Favicon and share image</t>
   </si>
   <si>
     <t>Blocked - still the platform placeholders</t>
   </si>
   <si>
-    <t>Remaining five service pages</t>
-  </si>
-  <si>
-    <t>Blocked - waiting on the Services-02 to 06 documents</t>
+    <t>Image optimisation</t>
+  </si>
+  <si>
+    <t>Service artwork is large; convert to WebP and lazy load</t>
+  </si>
+  <si>
+    <t>Open</t>
   </si>
   <si>
     <t>Dead code cleanup</t>
   </si>
   <si>
-    <t>Details.jsx, ServiceDetails.jsx, Projects, Counters, Testimonials and unused assets</t>
-  </si>
-  <si>
-    <t>Open</t>
-  </si>
-  <si>
-    <t>Image optimisation</t>
-  </si>
-  <si>
-    <t>about-enpro.jpeg is 519 KB; convert to WebP and add lazy loading</t>
+    <t>Details.jsx, ServiceDetails.jsx, Projects, Counters, Testimonials</t>
   </si>
 </sst>
 </file>
@@ -744,7 +813,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -770,6 +839,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -788,10 +860,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1133,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2498,16 +2570,302 @@
         <v>15</v>
       </c>
     </row>
+    <row r="53" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="H53" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H54" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H55" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="H56" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H57" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H58" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="H59" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="H60" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H61" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H62" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H63" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H52"/>
+  <autoFilter ref="A1:H63"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2516,21 +2874,21 @@
     <col min="5" max="5" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" ht="26" customHeight="1" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>172</v>
+      <c r="B1" s="10" t="s">
+        <v>199</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2538,33 +2896,33 @@
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>173</v>
+        <v>203</v>
       </c>
       <c r="C2" s="8">
         <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>174</v>
+        <v>204</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>175</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="C3" s="12">
+      <c r="B3" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="C3" s="13">
         <v>0</v>
       </c>
-      <c r="D3" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>175</v>
+      <c r="D3" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2572,57 +2930,74 @@
         <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>178</v>
+        <v>208</v>
       </c>
       <c r="C4" s="8">
         <v>27</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>179</v>
+        <v>209</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>180</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="C5" s="12">
+      <c r="B5" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="C5" s="13">
         <v>9</v>
       </c>
-      <c r="D5" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>183</v>
+      <c r="D5" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C6" s="13">
+        <v>11</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="2" width="78" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>184</v>
+        <v>217</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>185</v>
+        <v>218</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -2630,167 +3005,123 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>186</v>
+        <v>219</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>188</v>
+        <v>220</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>189</v>
+        <v>221</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>188</v>
+        <v>220</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>191</v>
+        <v>222</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>188</v>
+        <v>223</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>193</v>
+        <v>224</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>188</v>
+        <v>225</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>195</v>
+        <v>227</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>197</v>
+        <v>228</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>198</v>
+        <v>230</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>200</v>
+        <v>231</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>201</v>
+        <v>232</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>202</v>
+        <v>233</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>203</v>
+        <v>234</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>200</v>
+        <v>235</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>205</v>
+        <v>236</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>206</v>
+        <v>237</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>207</v>
+        <v>238</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>200</v>
+        <v>239</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>209</v>
+        <v>241</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>217</v>
+        <v>242</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild work log summary and add August month sheet
</commit_message>
<xml_diff>
--- a/Enpro-Daily-Work-Log.xlsx
+++ b/Enpro-Daily-Work-Log.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Daily Log" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Daily Summary" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Next Up" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="Next Up" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="Daily Summary" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="August 2026" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="309">
   <si>
     <t>Date</t>
   </si>
@@ -672,6 +673,84 @@
     <t>Whole project</t>
   </si>
   <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Landing page</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>About Us page</t>
+  </si>
+  <si>
+    <t>All six service detail pages</t>
+  </si>
+  <si>
+    <t>Built from the client's Rev-B documents</t>
+  </si>
+  <si>
+    <t>Client confirmations</t>
+  </si>
+  <si>
+    <t>Brand red kept for the environmental page, the service order, and the sections we added</t>
+  </si>
+  <si>
+    <t>To confirm</t>
+  </si>
+  <si>
+    <t>Contact form backend</t>
+  </si>
+  <si>
+    <t>Blocked - waiting on the destination email address</t>
+  </si>
+  <si>
+    <t>Blocked</t>
+  </si>
+  <si>
+    <t>Logo source file</t>
+  </si>
+  <si>
+    <t>Blocked - vector or transparent PNG needed</t>
+  </si>
+  <si>
+    <t>Social profile URLs</t>
+  </si>
+  <si>
+    <t>Blocked - all three links are placeholders</t>
+  </si>
+  <si>
+    <t>Phone number and address</t>
+  </si>
+  <si>
+    <t>Blocked - only the email address is available</t>
+  </si>
+  <si>
+    <t>Favicon and share image</t>
+  </si>
+  <si>
+    <t>Blocked - still the platform placeholders</t>
+  </si>
+  <si>
+    <t>Image optimisation</t>
+  </si>
+  <si>
+    <t>Service artwork is large; convert to WebP and lazy load</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>Dead code cleanup</t>
+  </si>
+  <si>
+    <t>Details.jsx, ServiceDetails.jsx, Projects, Counters, Testimonials</t>
+  </si>
+  <si>
     <t>Sessions</t>
   </si>
   <si>
@@ -687,22 +766,19 @@
     <t>2 (night + evening)</t>
   </si>
   <si>
-    <t>Landing page completed end to end, Services detail page built, About Us page rebuilt, 7 bugs fixed, full responsive pass</t>
+    <t>Landing page rebuilt end to end, Services detail page and About Us page created, seven production bugs fixed, full responsive pass</t>
   </si>
   <si>
     <t>~78%</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
     <t>No work</t>
   </si>
   <si>
     <t>3 (afternoon, evening, night)</t>
   </si>
   <si>
-    <t>Responsive overhaul, three sections redesigned, CTA and 404 rebuilt, documents re-verified, then a full round of client-requested refinements and the new photography put to use</t>
+    <t>Responsive overhaul across every page, three sections redesigned, CTA and 404 rebuilt, all three client documents re-verified, README written, work committed and pushed</t>
   </si>
   <si>
     <t>~88%</t>
@@ -711,116 +787,167 @@
     <t>1 (late night)</t>
   </si>
   <si>
-    <t>A round of client-requested refinements to the side menu, section labels and remaining numbers</t>
+    <t>Client refinements to the side menu, section labels, icons and hero slideshow</t>
   </si>
   <si>
     <t>~89%</t>
   </si>
   <si>
-    <t>1 (evening)</t>
-  </si>
-  <si>
-    <t>All five remaining service detail pages built from the client's documents, with per-service banners, photography and icons</t>
-  </si>
-  <si>
-    <t>~95%</t>
-  </si>
-  <si>
-    <t>15-Aug-2026 (cont.)</t>
-  </si>
-  <si>
-    <t>1 (night)</t>
-  </si>
-  <si>
-    <t>Client feedback round: green artwork for the environmental service, icon and spacing changes, blank-section fix, and a full cleanup</t>
+    <t>2 (evening + night)</t>
+  </si>
+  <si>
+    <t>All five remaining service detail pages built from the client's documents; client feedback round on icons, spacing and artwork; blank-section bug fixed; project cleaned up by about 17 MB</t>
   </si>
   <si>
     <t>~96%</t>
   </si>
   <si>
-    <t>Item</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Landing page</t>
-  </si>
-  <si>
-    <t>Complete</t>
-  </si>
-  <si>
-    <t>About Us page</t>
-  </si>
-  <si>
-    <t>All six service detail pages</t>
-  </si>
-  <si>
-    <t>Built from the client's Rev-B documents</t>
-  </si>
-  <si>
-    <t>Client confirmations</t>
-  </si>
-  <si>
-    <t>Brand red kept for the environmental page, the service order, and the sections we added</t>
-  </si>
-  <si>
-    <t>To confirm</t>
-  </si>
-  <si>
-    <t>Contact form backend</t>
-  </si>
-  <si>
-    <t>Blocked - waiting on the destination email address</t>
-  </si>
-  <si>
-    <t>Blocked</t>
-  </si>
-  <si>
-    <t>Logo source file</t>
-  </si>
-  <si>
-    <t>Blocked - vector or transparent PNG needed</t>
-  </si>
-  <si>
-    <t>Social profile URLs</t>
-  </si>
-  <si>
-    <t>Blocked - all three links are placeholders</t>
-  </si>
-  <si>
-    <t>Phone number and address</t>
-  </si>
-  <si>
-    <t>Blocked - only the email address is available</t>
-  </si>
-  <si>
-    <t>Favicon and share image</t>
-  </si>
-  <si>
-    <t>Blocked - still the platform placeholders</t>
-  </si>
-  <si>
-    <t>Image optimisation</t>
-  </si>
-  <si>
-    <t>Service artwork is large; convert to WebP and lazy load</t>
-  </si>
-  <si>
-    <t>Open</t>
-  </si>
-  <si>
-    <t>Dead code cleanup</t>
-  </si>
-  <si>
-    <t>Details.jsx, ServiceDetails.jsx, Projects, Counters, Testimonials</t>
+    <t>ENPRO WEBSITE — AUGUST 2026</t>
+  </si>
+  <si>
+    <t>Categories</t>
+  </si>
+  <si>
+    <t>What was done</t>
+  </si>
+  <si>
+    <t>01-Aug</t>
+  </si>
+  <si>
+    <t>Worked</t>
+  </si>
+  <si>
+    <t>Bug Fix, Development, Fix, Responsive</t>
+  </si>
+  <si>
+    <t>02-Aug</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>03-Aug</t>
+  </si>
+  <si>
+    <t>Assets, Client Changes, Delivery, Design, Reporting, Responsive, Review</t>
+  </si>
+  <si>
+    <t>04-Aug</t>
+  </si>
+  <si>
+    <t>Client Changes, Consistency</t>
+  </si>
+  <si>
+    <t>05-Aug</t>
+  </si>
+  <si>
+    <t>Wednesday</t>
+  </si>
+  <si>
+    <t>06-Aug</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>07-Aug</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>08-Aug</t>
+  </si>
+  <si>
+    <t>09-Aug</t>
+  </si>
+  <si>
+    <t>10-Aug</t>
+  </si>
+  <si>
+    <t>11-Aug</t>
+  </si>
+  <si>
+    <t>12-Aug</t>
+  </si>
+  <si>
+    <t>13-Aug</t>
+  </si>
+  <si>
+    <t>14-Aug</t>
+  </si>
+  <si>
+    <t>15-Aug</t>
+  </si>
+  <si>
+    <t>Cleanup, Content, Design, Development, Fix, Quality</t>
+  </si>
+  <si>
+    <t>16-Aug</t>
+  </si>
+  <si>
+    <t>17-Aug</t>
+  </si>
+  <si>
+    <t>18-Aug</t>
+  </si>
+  <si>
+    <t>19-Aug</t>
+  </si>
+  <si>
+    <t>20-Aug</t>
+  </si>
+  <si>
+    <t>21-Aug</t>
+  </si>
+  <si>
+    <t>22-Aug</t>
+  </si>
+  <si>
+    <t>23-Aug</t>
+  </si>
+  <si>
+    <t>24-Aug</t>
+  </si>
+  <si>
+    <t>25-Aug</t>
+  </si>
+  <si>
+    <t>26-Aug</t>
+  </si>
+  <si>
+    <t>27-Aug</t>
+  </si>
+  <si>
+    <t>28-Aug</t>
+  </si>
+  <si>
+    <t>29-Aug</t>
+  </si>
+  <si>
+    <t>30-Aug</t>
+  </si>
+  <si>
+    <t>31-Aug</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>4 days</t>
+  </si>
+  <si>
+    <t>Landing page, About Us page and all six service detail pages delivered — project at ~96%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -843,6 +970,18 @@
     <font>
       <b/>
       <color rgb="FF15803D"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <color rgb="FF9CA3AF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
   <fills count="6">
@@ -885,7 +1024,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -914,6 +1053,18 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -926,17 +1077,20 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3145,137 +3299,139 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="4" max="4" width="82" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="5" max="5" width="86" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" ht="26" customHeight="1" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>220</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="C2" s="8">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="D2" s="8">
         <v>14</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
+      <c r="E2" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="C3" s="13">
+      <c r="B3" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="17">
         <v>0</v>
       </c>
-      <c r="D3" s="12" t="s">
-        <v>227</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E3" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="C4" s="8">
+        <v>65</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="D4" s="8">
         <v>27</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+      <c r="E4" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="B5" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="C5" s="13">
+      <c r="B5" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="D5" s="17">
         <v>9</v>
       </c>
-      <c r="D5" s="12" t="s">
-        <v>232</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="E5" s="16" t="s">
+        <v>257</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="C6" s="13">
-        <v>11</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>235</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>237</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="C7" s="13">
-        <v>8</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>239</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>240</v>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D6" s="8">
+        <v>19</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>261</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
@@ -3291,10 +3447,10 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>241</v>
+        <v>219</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>7</v>
@@ -3302,127 +3458,818 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>243</v>
+        <v>221</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>244</v>
+        <v>222</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>245</v>
+        <v>223</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>244</v>
+        <v>222</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>246</v>
+        <v>224</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>244</v>
+        <v>225</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>250</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>251</v>
+        <v>229</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>253</v>
+        <v>230</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>255</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>253</v>
+        <v>233</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>256</v>
+        <v>234</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>253</v>
+        <v>235</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>258</v>
+        <v>236</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>253</v>
+        <v>237</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>260</v>
+        <v>238</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>261</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>253</v>
+        <v>239</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>263</v>
+        <v>241</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>264</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>265</v>
+        <v>243</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>266</v>
+        <v>244</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>264</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="62" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>265</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>266</v>
+      </c>
+      <c r="D3" s="17">
+        <v>14</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>266</v>
+      </c>
+      <c r="D5" s="17">
+        <v>27</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
+        <v>273</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>266</v>
+      </c>
+      <c r="D6" s="17">
+        <v>9</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>274</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>266</v>
+      </c>
+      <c r="D17" s="17">
+        <v>19</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>289</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>298</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>305</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="21" t="s">
+        <v>306</v>
+      </c>
+      <c r="B35" s="21" t="s">
+        <v>269</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>307</v>
+      </c>
+      <c r="D35" s="22">
+        <v>69</v>
+      </c>
+      <c r="E35" s="21" t="s">
+        <v>269</v>
+      </c>
+      <c r="F35" s="21" t="s">
+        <v>308</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>